<commit_message>
chore: initial repository scaffolding and PBL documentation
</commit_message>
<xml_diff>
--- a/submission_reports/Java_PBL_RAG_Work_Logs.xlsx
+++ b/submission_reports/Java_PBL_RAG_Work_Logs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\Lenovo\OneDrive\Desktop\RAG\submission_reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D631148D-6BA0-4BCA-879E-E3EB8DCDB95B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E1BED97E-037C-4FB2-8A55-160260181BA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{3A504E05-BC5F-4434-86F1-90D18B3D4833}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{D4EA71C4-BF1A-4DE3-B473-324BE1EC24B0}"/>
   </bookViews>
   <sheets>
     <sheet name="Daily Work Log" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1827" uniqueCount="538">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1827" uniqueCount="537">
   <si>
     <t>Date</t>
   </si>
@@ -58,7 +58,7 @@
     <t>Work Description (What did you do today?)</t>
   </si>
   <si>
-    <t>Aryan Kumar Singh</t>
+    <t>Shaurya Dixit</t>
   </si>
   <si>
     <t>Module 1: Core RAG Engine &amp; LLM Orchestration</t>
@@ -67,232 +67,232 @@
     <t>Completed</t>
   </si>
   <si>
-    <t>Finalized project topic on RAG using Spring Boot &amp; Neon PostgreSQL; drafted project abstract with Guide Er. Ram Babu Buri.</t>
-  </si>
-  <si>
-    <t>Awantika Jaiswal</t>
-  </si>
-  <si>
-    <t>Module 2: Document Ingestion, Parsing &amp; Chunking</t>
-  </si>
-  <si>
-    <t>Researched unstructured document processing standards (PDF, DOCX, TXT) suitable for enterprise RAG pipelines.</t>
-  </si>
-  <si>
-    <t>Devansh Maini</t>
+    <t>Finalized RAG architecture with Guide Er. Ram Babu Buri; drafted project abstract and registration.</t>
+  </si>
+  <si>
+    <t>Yashvardhan Singh Chauhan</t>
+  </si>
+  <si>
+    <t>Module 2: Document Ingestion, Parsing &amp; Chunking (Kaggle Dataset)</t>
+  </si>
+  <si>
+    <t>Researched Kaggle academic paper datasets (arXiv CS AI/ML corpus) for document extraction.</t>
+  </si>
+  <si>
+    <t>Vaibhav Tank</t>
   </si>
   <si>
     <t>Module 3: Neon PostgreSQL Vector Store &amp; Spring Security</t>
   </si>
   <si>
-    <t>Researched PostgreSQL vector extensions (pgvector) and Neon serverless database deployment models.</t>
-  </si>
-  <si>
-    <t>Aviral Joshi</t>
+    <t>Researched PostgreSQL pgvector extension and Neon serverless database deployment.</t>
+  </si>
+  <si>
+    <t>Rajveer Singh Ranawat</t>
   </si>
   <si>
     <t>Module 4: React TypeScript UI &amp; Electron Desktop Integration</t>
   </si>
   <si>
-    <t>Researched Electron with React + TypeScript integration patterns for cross-platform desktop delivery.</t>
-  </si>
-  <si>
-    <t>Akshita Mawaliya</t>
-  </si>
-  <si>
-    <t>Module 5: RAG Triad Evaluation, Analytics &amp; Testing</t>
-  </si>
-  <si>
-    <t>Researched RAG evaluation methodologies (Ragas, TruLens, RAG Triad: Context Relevance, Groundedness, Answer Relevance).</t>
-  </si>
-  <si>
-    <t>Convened team kickoff meeting; mapped out 5-module architectural breakdown and GitHub repository strategy.</t>
-  </si>
-  <si>
-    <t>Evaluated Apache Tika vs PDFBox Java libraries for token-safe document text extraction.</t>
-  </si>
-  <si>
-    <t>Created Neon DB cloud account; provisioned development instance and tested remote JDBC connectivity.</t>
-  </si>
-  <si>
-    <t>Evaluated UI design frameworks (Tailwind CSS, Shadcn-UI) for responsive dark/light mode desktop client.</t>
-  </si>
-  <si>
-    <t>Studied JUnit 5, Mockito, and Testcontainers setup for Spring Boot integration testing.</t>
-  </si>
-  <si>
-    <t>Established GitHub organization repo and initialized branch policies (min 3 commits/student per week).</t>
-  </si>
-  <si>
-    <t>Defined Document Ingestion module boundary and input format specifications.</t>
-  </si>
-  <si>
-    <t>Evaluated Spring Boot PostgreSQL drivers and pgvector vector type compatibility.</t>
-  </si>
-  <si>
-    <t>Drafted wireframe sketches for Chat interface, Document Management panel, and System Settings.</t>
-  </si>
-  <si>
-    <t>Drafted quality assurance guidelines and test coverage targets for all 5 team modules.</t>
-  </si>
-  <si>
-    <t>Drafted high-level system context diagram and RAG orchestration lifecycle.</t>
-  </si>
-  <si>
-    <t>Created initial technical notes on text pre-processing and metadata sanitization.</t>
-  </si>
-  <si>
-    <t>Drafted schema concepts for user authentication, roles, document metadata, and embedding chunks.</t>
-  </si>
-  <si>
-    <t>Researched Electron IPC (Inter-Process Communication) security best practices (contextIsolation, preload).</t>
-  </si>
-  <si>
-    <t>Created evaluation metric formula sheet for measuring hallucination rates and retrieval latency.</t>
-  </si>
-  <si>
-    <t>Attended Saturday mentor review; presented project abstract and incorporated mentor feedback on vector store scope.</t>
-  </si>
-  <si>
-    <t>Participated in mentor review meeting; aligned document processing inputs with team vector store schema.</t>
-  </si>
-  <si>
-    <t>Participated in mentor meeting; validated database performance objectives with mentor.</t>
-  </si>
-  <si>
-    <t>Participated in mentor meeting; demonstrated UI mockup ideas to mentor Er. Ram Babu Buri.</t>
-  </si>
-  <si>
-    <t>Participated in mentor meeting; reviewed testing and evaluation criteria with mentor.</t>
-  </si>
-  <si>
-    <t>Synthesized mentor notes, aligned team deliverables for upcoming SRS milestone.</t>
-  </si>
-  <si>
-    <t>Organized technical documentation notes and prepared next week's parser requirements.</t>
-  </si>
-  <si>
-    <t>Documented database connection pooling benchmarks (HikariCP) for Neon serverless.</t>
-  </si>
-  <si>
-    <t>Refined UI wireframe feedback and documented desktop packaging requirements.</t>
-  </si>
-  <si>
-    <t>Finalized week 1 log summary and set up evaluation documentation repository.</t>
-  </si>
-  <si>
-    <t>Formulated Functional Requirements for Core RAG Service (query embedding, prompt construction, LLM response stream).</t>
-  </si>
-  <si>
-    <t>Authored SRS Functional Requirements for Document Ingestion (multi-file upload, MIME detection, text extraction).</t>
-  </si>
-  <si>
-    <t>Authored SRS Data Requirements: PostgreSQL 16 schema, pgvector vector(1536) column requirements.</t>
-  </si>
-  <si>
-    <t>Authored SRS User Interface Requirements: Electron desktop frame, React responsive layouts, accessibility.</t>
-  </si>
-  <si>
-    <t>Authored SRS Testing &amp; Verification Requirements: unit test coverage (&gt;80%), end-to-end integration tests.</t>
-  </si>
-  <si>
-    <t>Defined Non-Functional Requirements: retrieval latency (&lt;200ms), concurrent query handling, error fallback.</t>
-  </si>
-  <si>
-    <t>Specified chunking requirements: recursive splitting, token boundaries (512 tokens), 10% overlap strategy.</t>
-  </si>
-  <si>
-    <t>Defined Security Requirements: JWT token authentication, bcrypt password hashing, CORS policies, Role-Based Access.</t>
-  </si>
-  <si>
-    <t>Specified real-time chat streaming UI requirements, code block syntax highlighting, markdown rendering.</t>
-  </si>
-  <si>
-    <t>Specified RAG Triad evaluation metrics requirements: Context Recall, Context Precision, Answer Faithfulness.</t>
-  </si>
-  <si>
-    <t>Authored SRS Section 2: Overall System Description, User Characteristics, and Operating Environment.</t>
-  </si>
-  <si>
-    <t>Defined error handling requirements for corrupted PDFs, password-protected files, and unsupported formats.</t>
-  </si>
-  <si>
-    <t>Documented database performance metrics: HNSW indexing vs IVFFlat trade-offs for Neon cloud storage.</t>
-  </si>
-  <si>
-    <t>Defined desktop client offline behavior, local cached credentials, and API connection indicator.</t>
+    <t>Researched Electron 30 with React 18 and TypeScript for cross-platform desktop delivery.</t>
+  </si>
+  <si>
+    <t>Yashpal Singh Bhati</t>
+  </si>
+  <si>
+    <t>Module 5: RAG Triad Evaluation, Performance Analytics &amp; Testing</t>
+  </si>
+  <si>
+    <t>Researched RAG Triad evaluation metrics (Context Relevance, Faithfulness, Answer Relevance).</t>
+  </si>
+  <si>
+    <t>Convened kickoff meeting; defined 5-module boundaries and GitHub workflow for team.</t>
+  </si>
+  <si>
+    <t>Evaluated Apache Tika and PDFBox libraries for handling complex Kaggle research paper PDFs.</t>
+  </si>
+  <si>
+    <t>Provisioned Neon PostgreSQL development instance and verified remote JDBC connectivity.</t>
+  </si>
+  <si>
+    <t>Evaluated Tailwind CSS and Lucide icons for dark-mode responsive UI design.</t>
+  </si>
+  <si>
+    <t>Evaluated JUnit 5, Mockito, and Testcontainers setup for Spring Boot automated testing.</t>
+  </si>
+  <si>
+    <t>Established repository branching policy (minimum 3 commits/student/week) on GitHub.</t>
+  </si>
+  <si>
+    <t>Defined Document Ingestion module boundary and input MIME format validation standards.</t>
+  </si>
+  <si>
+    <t>Evaluated Spring Boot pgvector drivers and HNSW vector index compatibility.</t>
+  </si>
+  <si>
+    <t>Drafted wireframe layouts for Chat Canvas, Citation Inspector, and Ingestion Panel.</t>
+  </si>
+  <si>
+    <t>Drafted QA test coverage targets (&gt;80%) and golden dataset validation plan.</t>
+  </si>
+  <si>
+    <t>Drafted high-level RAG orchestration flow and context assembly specifications.</t>
+  </si>
+  <si>
+    <t>Analyzed mathematical equations and two-column layout parsing challenges in academic papers.</t>
+  </si>
+  <si>
+    <t>Drafted relational schemas for user authentication, roles, document metadata, and chunks.</t>
+  </si>
+  <si>
+    <t>Researched Electron IPC security best practices (contextIsolation, sandboxed preload).</t>
+  </si>
+  <si>
+    <t>Formulated mathematical evaluation formulas for measuring hallucination rates.</t>
+  </si>
+  <si>
+    <t>Attended Saturday mentor review; defended architectural scope with Er. Ram Babu Buri.</t>
+  </si>
+  <si>
+    <t>Participated in Saturday mentor review; confirmed Kaggle dataset curation parameters.</t>
+  </si>
+  <si>
+    <t>Attended Saturday mentor review; presented database connection pooling architecture.</t>
+  </si>
+  <si>
+    <t>Demonstrated UI wireframe concepts to mentor Er. Ram Babu Buri during Saturday review.</t>
+  </si>
+  <si>
+    <t>Participated in Saturday mentor review; discussed evaluation criteria with mentor.</t>
+  </si>
+  <si>
+    <t>Compiled mentor notes and aligned week 2 SRS deliverables with team.</t>
+  </si>
+  <si>
+    <t>Documented text normalization rules and prepared next week's parser requirements.</t>
+  </si>
+  <si>
+    <t>Documented database performance objectives and connection limits in Neon.</t>
+  </si>
+  <si>
+    <t>Documented desktop client packaging and performance requirements.</t>
+  </si>
+  <si>
+    <t>Established testing directory structure and test metrics documentation repository.</t>
+  </si>
+  <si>
+    <t>Authored SRS Functional Requirements for Core RAG Service (query embedding, prompt assembly, SSE stream).</t>
+  </si>
+  <si>
+    <t>Authored SRS Functional Requirements for Ingestion (Kaggle dataset multi-file upload, Tika extraction).</t>
+  </si>
+  <si>
+    <t>Authored SRS Data Requirements: PostgreSQL 16 schema, pgvector vector(1536) columns.</t>
+  </si>
+  <si>
+    <t>Authored SRS User Interface Requirements: Electron desktop shell, React responsive layout.</t>
+  </si>
+  <si>
+    <t>Authored SRS Testing Requirements: unit test coverage (&gt;80%), end-to-end integration tests.</t>
+  </si>
+  <si>
+    <t>Specified non-functional performance requirements: retrieval latency &lt;120ms, error fallback.</t>
+  </si>
+  <si>
+    <t>Specified chunking requirements: recursive splitting, 500-token window, 50-token overlap.</t>
+  </si>
+  <si>
+    <t>Defined Security Requirements: JWT HMAC-SHA256 tokens, BCrypt password hashing, RBAC.</t>
+  </si>
+  <si>
+    <t>Specified real-time chat streaming UI, code block syntax highlighting, and markdown rendering.</t>
+  </si>
+  <si>
+    <t>Specified RAG Triad evaluation metrics requirements: Context Recall, Precision, Faithfulness.</t>
+  </si>
+  <si>
+    <t>Authored SRS Section 2: Overall System Description and Operating Environment.</t>
+  </si>
+  <si>
+    <t>Defined error handling requirements for corrupted files, scanned PDFs, and oversized uploads.</t>
+  </si>
+  <si>
+    <t>Documented HNSW index parameters (m=16, ef_construction=64) on Neon serverless.</t>
+  </si>
+  <si>
+    <t>Defined desktop client offline behavior, local cached credentials, and network indicators.</t>
   </si>
   <si>
     <t>Defined compliance checklist for IEEE 830 standards across all 5 modules.</t>
   </si>
   <si>
-    <t>Specified REST API contract for query endpoint (/api/rag/chat) and SSE streaming (/api/rag/stream).</t>
-  </si>
-  <si>
-    <t>Specified asynchronous document parsing job status lifecycle (PENDING, PROCESSING, INDEXED, FAILED).</t>
-  </si>
-  <si>
-    <t>Specified audit logging requirements for user queries, document uploads, and administrative actions.</t>
+    <t>Specified REST API contract for /api/rag/chat and Server-Sent Events streaming.</t>
+  </si>
+  <si>
+    <t>Specified asynchronous job tracking status lifecycle (UPLOADED -&gt; PARSING -&gt; INDEXED).</t>
+  </si>
+  <si>
+    <t>Specified audit logging requirements for user queries, tokens used, and upload timestamps.</t>
   </si>
   <si>
     <t>Drafted UI navigation hierarchy and screen transition specifications.</t>
   </si>
   <si>
-    <t>Compiled individual module SRS sections into cohesive 35-page master SRS document.</t>
-  </si>
-  <si>
-    <t>Attended Saturday mentor review with SRS draft; reviewed RAG API specifications with mentor.</t>
-  </si>
-  <si>
-    <t>Attended mentor review; defended parsing throughput and file size limitation parameters (max 25MB).</t>
-  </si>
-  <si>
-    <t>Presented database and security section to mentor during Saturday review meeting.</t>
-  </si>
-  <si>
-    <t>Reviewed UI SRS requirements with mentor; received approval on split-pane desktop workspace layout.</t>
-  </si>
-  <si>
-    <t>Presented quality assurance and evaluation criteria during mentor meeting.</t>
-  </si>
-  <si>
-    <t>Incorporated mentor suggestions regarding fallback when vector search similarity score is below threshold.</t>
-  </si>
-  <si>
-    <t>Updated document ingestion requirements matrix in SRS master document.</t>
-  </si>
-  <si>
-    <t>Finalized database capacity planning and Neon auto-scaling constraints in SRS.</t>
-  </si>
-  <si>
-    <t>Refined desktop application performance requirements (RAM consumption &lt;150MB in idle state).</t>
-  </si>
-  <si>
-    <t>Created SRS traceability matrix mapping requirements to planned development milestones.</t>
-  </si>
-  <si>
-    <t>Drafted system-level Use Case Diagram mapping Actors (Student, Researcher, Admin) to RAG actions.</t>
-  </si>
-  <si>
-    <t>Designed Sequence Diagram for Document Ingestion: Upload -&gt; MIME Validator -&gt; Parser -&gt; Chunker -&gt; Embedding Service.</t>
-  </si>
-  <si>
-    <t>Designed Entity-Relationship (ER) Diagram: Users, Roles, Documents, DocumentChunks (with vector embeddings), AuditLogs.</t>
-  </si>
-  <si>
-    <t>Designed Component Diagram showing Electron Main Process, Preload Bridge, React Renderer, and HTTP/SSE Client.</t>
-  </si>
-  <si>
-    <t>Designed Sequence Diagram for Automated RAG Evaluation Pipeline (Test Runner -&gt; Triad Evaluator -&gt; Metrics DB).</t>
-  </si>
-  <si>
-    <t>Designed Sequence Diagram for RAG Query Processing: User -&gt; Electron UI -&gt; Spring Boot -&gt; Neon pgvector -&gt; LLM -&gt; Client.</t>
-  </si>
-  <si>
-    <t>Constructed Class Diagram for DocumentParserFactory, TikaParserImpl, PdfBoxParserImpl, and RecursiveChunker.</t>
-  </si>
-  <si>
-    <t>Constructed Class Diagram for JPA entities: UserEntity, RoleEntity, DocumentEntity, ChunkEntity.</t>
+    <t>Compiled individual module SRS sections into unified 35-page master SRS document.</t>
+  </si>
+  <si>
+    <t>Attended Saturday mentor review; reviewed RAG functional specifications with mentor.</t>
+  </si>
+  <si>
+    <t>Attended Saturday mentor review; defended parsing throughput and file size constraints (25MB).</t>
+  </si>
+  <si>
+    <t>Presented database and security section to mentor during Saturday review.</t>
+  </si>
+  <si>
+    <t>Reviewed UI SRS requirements with mentor; received approval on split-pane workspace layout.</t>
+  </si>
+  <si>
+    <t>Presented quality assurance and evaluation criteria during Saturday review.</t>
+  </si>
+  <si>
+    <t>Incorporated mentor suggestions on similarity confidence threshold filtering.</t>
+  </si>
+  <si>
+    <t>Updated document ingestion requirements matrix in master SRS document.</t>
+  </si>
+  <si>
+    <t>Finalized Neon database capacity planning and SSL/TLS constraints in SRS.</t>
+  </si>
+  <si>
+    <t>Refined desktop application performance requirements (RAM consumption &lt;150MB).</t>
+  </si>
+  <si>
+    <t>Created SRS traceability matrix mapping requirements to development milestones.</t>
+  </si>
+  <si>
+    <t>Drafted system-level Use Case Diagram mapping Actors (Student, Researcher, Admin) to actions.</t>
+  </si>
+  <si>
+    <t>Designed Sequence Diagram for Kaggle Ingestion: Upload -&gt; MIME Validator -&gt; Parser -&gt; Chunker.</t>
+  </si>
+  <si>
+    <t>Designed Entity-Relationship (ER) Diagram: Users, Roles, Documents, DocumentChunks, AuditLogs.</t>
+  </si>
+  <si>
+    <t>Designed Component Diagram showing Electron Main, Preload Bridge, React Renderer, and SSE Client.</t>
+  </si>
+  <si>
+    <t>Designed Sequence Diagram for Automated RAG Evaluation Pipeline (Test Runner -&gt; Triad Evaluator).</t>
+  </si>
+  <si>
+    <t>Designed Sequence Diagram for RAG Query Processing: User -&gt; Electron -&gt; Spring Boot -&gt; Neon -&gt; LLM.</t>
+  </si>
+  <si>
+    <t>Constructed Class Diagram for DocumentParser, TikaParserImpl, and RecursiveTextChunker.</t>
+  </si>
+  <si>
+    <t>Constructed Class Diagram for JPA entities: User, Role, Document, DocumentChunk.</t>
   </si>
   <si>
     <t>Constructed Sequence Diagram for desktop file drag-and-drop ingestion to Spring Boot API.</t>
@@ -301,22 +301,22 @@
     <t>Constructed Component Diagram for Test Automation and Telemetry collector in Spring Boot.</t>
   </si>
   <si>
-    <t>Constructed Class Diagram for RagOrchestrationService, PromptTemplateBuilder, and LlmClientAdapter.</t>
-  </si>
-  <si>
-    <t>Modeled State Machine Diagram for DocumentStatus (UPLOADED -&gt; PARSING -&gt; CHUNKED -&gt; EMBEDDED -&gt; READY).</t>
-  </si>
-  <si>
-    <t>Designed Sequence Diagram for User Authentication and JWT verification filter chain in Spring Security.</t>
-  </si>
-  <si>
-    <t>Modeled UI State Flow Diagram: Auth Guard -&gt; Workspace Selection -&gt; Chat Session -&gt; Source Inspector.</t>
+    <t>Constructed Class Diagram for RagOrchestrationService, PromptTemplateBuilder, and ChatClient.</t>
+  </si>
+  <si>
+    <t>Modeled State Machine Diagram for DocumentStatus (UPLOADED -&gt; PARSING -&gt; CHUNKED -&gt; INDEXED).</t>
+  </si>
+  <si>
+    <t>Designed Sequence Diagram for User Authentication and JWT verification filter chain.</t>
+  </si>
+  <si>
+    <t>Modeled UI State Flow Diagram: Auth Guard -&gt; Workspace Selection -&gt; Chat Session -&gt; Citations.</t>
   </si>
   <si>
     <t>Created UML Traceability Matrix cross-referencing SRS functional requirements to UML classes.</t>
   </si>
   <si>
-    <t>Modeled State Machine Diagram for conversational session lifecycle and context cache.</t>
+    <t>Modeled State Machine Diagram for conversational session lifecycle and context budgeting.</t>
   </si>
   <si>
     <t>Designed Activity Diagram illustrating token-aware recursive text splitting with sliding window.</t>
@@ -325,7 +325,7 @@
     <t>Modeled database physical deployment schema with Neon connection pooler and pgvector extension.</t>
   </si>
   <si>
-    <t>Designed Class/Interface Diagram for React State Stores (Zustand: useChatStore, useDocStore, useAuthStore).</t>
+    <t>Designed Class/Interface Diagram for React State Stores (useChatStore, useDocStore).</t>
   </si>
   <si>
     <t>Drafted Deployment Diagram showing Client Electron App, Cloud Spring Boot Service, and Neon DB.</t>
@@ -337,7 +337,7 @@
     <t>Reviewed Ingestion UML models with mentor; clarified multipart file streaming boundary.</t>
   </si>
   <si>
-    <t>Presented ER diagram and database security sequence diagrams to mentor during Saturday review.</t>
+    <t>Presented ER diagram and security sequence diagrams to mentor during Saturday review.</t>
   </si>
   <si>
     <t>Reviewed Electron architectural component diagram with mentor; confirmed IPC security boundaries.</t>
@@ -346,13 +346,13 @@
     <t>Presented overall deployment architecture and evaluation UML models in Saturday mentor review.</t>
   </si>
   <si>
-    <t>Refined Class Diagram methods based on mentor recommendations for dependency injection and loose coupling.</t>
+    <t>Refined Class Diagram methods based on mentor recommendations for loose coupling.</t>
   </si>
   <si>
     <t>Finalized document ingestion package diagram in UML specification document.</t>
   </si>
   <si>
-    <t>Adjusted foreign key cascading rules and chunk index structures per mentor input.</t>
+    <t>Adjusted foreign key cascading rules (ON DELETE CASCADE) per mentor input.</t>
   </si>
   <si>
     <t>Compiled UI design artifacts and component interaction specs into UML design report.</t>
@@ -361,7 +361,7 @@
     <t>Assembled all UML diagrams into Chapter 3 of Project Design Documentation.</t>
   </si>
   <si>
-    <t>Set up local development IDE (IntelliJ IDEA) with Spring Boot 3.3.x, Java 21, and Spring AI milestone dependencies.</t>
+    <t>Set up local IDE with Spring Boot 3.3, Java 21, and Spring AI milestone dependencies.</t>
   </si>
   <si>
     <t>Configured Maven dependencies for Apache Tika Core/Parsers and Apache PDFBox 3.x.</t>
@@ -376,28 +376,28 @@
     <t>Configured JUnit 5, AssertJ, and Mockito testing dependencies in Maven POM.</t>
   </si>
   <si>
-    <t>Created root Maven multi-module parent POM / project structure with defined member sub-modules.</t>
+    <t>Created root Maven multi-module parent POM structure with defined member sub-modules.</t>
+  </si>
+  <si>
+    <t>Downloaded sample research paper dataset from Kaggle (arXiv multi-domain corpus).</t>
+  </si>
+  <si>
+    <t>Authored DDL migration script: created tables users, roles, documents, document_chunks.</t>
+  </si>
+  <si>
+    <t>Set up Electron 30.x desktop scaffolding with secure contextIsolation and preload script.</t>
+  </si>
+  <si>
+    <t>Set up H2 in-memory test profile with pgvector mock functions for unit test runs.</t>
+  </si>
+  <si>
+    <t>Drafted Spring AI VectorStore interface abstraction and mock embedding generator.</t>
   </si>
   <si>
     <t>Created Git branch 'feature/member2-doc-ingestion' and committed base document model interfaces.</t>
   </si>
   <si>
-    <t>Authored DDL migration script 'V1__init_schema.sql': created tables users, roles, documents, document_chunks.</t>
-  </si>
-  <si>
-    <t>Set up Electron 30.x desktop scaffolding with secure contextIsolation and preload script.</t>
-  </si>
-  <si>
-    <t>Set up H2 in-memory test profile with pgvector mock functions for unit test runs.</t>
-  </si>
-  <si>
-    <t>Drafted Spring AI VectorStore interface abstraction and mock embedding generator for local testing.</t>
-  </si>
-  <si>
-    <t>Implemented unit prototype for PDF text extraction and verified handling of multi-page sample documents.</t>
-  </si>
-  <si>
-    <t>Created HNSW index on document_chunks(embedding vector_cosine_ops) for sub-millisecond similarity search.</t>
+    <t>Created HNSW index on document_chunks(embedding vector_cosine_ops) for sub-100ms similarity search.</t>
   </si>
   <si>
     <t>Created Git branch 'feature/member4-ui-electron' and pushed base desktop client skeleton.</t>
@@ -409,10 +409,10 @@
     <t>Configured application-dev.yml and environment variable templates for API keys and DB credentials.</t>
   </si>
   <si>
-    <t>Tested text boundary detection and cleaning of whitespace, headers, and footers.</t>
-  </si>
-  <si>
-    <t>Created Git branch 'feature/member3-database-security' and committed Flyway/Liquibase migration scripts.</t>
+    <t>Tested text boundary detection and cleaning of whitespace, headers, and footers on Kaggle papers.</t>
+  </si>
+  <si>
+    <t>Created Git branch 'feature/member3-database-security' and committed Flyway migration scripts.</t>
   </si>
   <si>
     <t>Built responsive UI layout: Collapsible Sidebar, Main Chat Canvas, Source Citation Drawer.</t>
@@ -421,10 +421,10 @@
     <t>Drafted automated test suites for verifying database schema integrity and constraints.</t>
   </si>
   <si>
-    <t>Attended Saturday mentor review; verified development toolchain and Maven build configurations with mentor.</t>
-  </si>
-  <si>
-    <t>Participated in mentor review; demonstrated prototype parsing results for complex academic PDFs.</t>
+    <t>Attended Saturday mentor review; verified development toolchain and Maven build with mentor.</t>
+  </si>
+  <si>
+    <t>Participated in mentor review; demonstrated prototype parsing results for complex Kaggle PDFs.</t>
   </si>
   <si>
     <t>Presented live Neon DB connection and vector table schema to mentor during review.</t>
@@ -451,10 +451,10 @@
     <t>Created GitHub Actions CI workflow draft for automated build verification on pull requests.</t>
   </si>
   <si>
-    <t>Implemented RagOrchestrationServiceImpl: handles incoming user query, generates query vector, queries vector store.</t>
-  </si>
-  <si>
-    <t>Implemented TikaDocumentParser: extracts clean text and metadata (author, title, page count) from PDF, DOCX, TXT.</t>
+    <t>Implemented RagOrchestrationServiceImpl: handles incoming query, generates query vector, queries vector store.</t>
+  </si>
+  <si>
+    <t>Implemented TikaDocumentParser: extracts clean text and metadata (author, title, page count) from Kaggle PDFs.</t>
   </si>
   <si>
     <t>Implemented Spring Security 6 security filter chain with stateless SessionCreationPolicy.STATELESS.</t>
@@ -505,7 +505,7 @@
     <t>Created AuthController with /api/auth/register and /api/auth/login endpoints with BCrypt password encoding.</t>
   </si>
   <si>
-    <t>Created ChatInput component with multi-line auto-resizing textarea and submit on Enter (Shift+Enter for newline).</t>
+    <t>Created ChatInput component with multi-line auto-resizing textarea and submit on Enter.</t>
   </si>
   <si>
     <t>Added Jacoco code coverage plugin to Maven build and generated initial coverage reports.</t>
@@ -541,7 +541,7 @@
     <t>Committed test suites to branch 'feature/member5-analytics-evaluation' (3 commits).</t>
   </si>
   <si>
-    <t>Integrated Spring AI EmbeddingModel client (configured for text-embedding-3-small / local BAAI embeddings).</t>
+    <t>Integrated Spring AI EmbeddingModel client (configured for text-embedding-3-small / local embeddings).</t>
   </si>
   <si>
     <t>Implemented DocumentUploadController with POST /api/documents/upload handling multipart file uploads.</t>
@@ -748,7 +748,7 @@
     <t>Implemented SystemSettings panel allowing configuration of Backend API URL, LLM model choice, and dark/light theme.</t>
   </si>
   <si>
-    <t>Created automated evaluation test runner with a golden dataset of 50 ground-truth Q&amp;A pairs.</t>
+    <t>Created automated evaluation test runner with a golden dataset of 50 ground-truth Q&amp;A pairs from Kaggle.</t>
   </si>
   <si>
     <t>Refactored PromptTemplateBuilder to inject explicit negative constraints ('Answer only from context, else state unknown').</t>
@@ -769,7 +769,7 @@
     <t>Added structured JSON output mode for programmatic Q&amp;A extraction.</t>
   </si>
   <si>
-    <t>Created sample dataset of 15 technical research papers and textbook chapters for system benchmark.</t>
+    <t>Curated Kaggle dataset benchmark of 25 technical research papers and textbook chapters for system benchmark.</t>
   </si>
   <si>
     <t>Optimized SQL query performance by adding composite index on document_chunks(document_id, chunk_index).</t>
@@ -814,7 +814,7 @@
     <t>Created 'develop' branch; orchestrated Pull Requests from all 5 feature branches and resolved merge conflicts.</t>
   </si>
   <si>
-    <t>Tested end-to-end document upload pipeline using 10 different PDF and DOCX documents via Electron UI.</t>
+    <t>Tested end-to-end document upload pipeline using 10 different Kaggle PDF documents via Electron UI.</t>
   </si>
   <si>
     <t>Configured production-grade CORS configuration in Spring Security allowing electron:// and localhost origins.</t>
@@ -904,7 +904,7 @@
     <t>Benchmarked Spring AI prompt throughput under concurrent load; optimized prompt string concatenation.</t>
   </si>
   <si>
-    <t>Benchmarked document parsing throughput under simultaneous multi-document uploads.</t>
+    <t>Benchmarked document parsing throughput under simultaneous multi-document uploads from Kaggle dataset.</t>
   </si>
   <si>
     <t>Configured Neon PgBouncer connection pooler in transaction mode for high concurrency support.</t>
@@ -994,7 +994,7 @@
     <t>Authored Project Report Chapter 1: Introduction, Problem Statement, Objectives, and Scope of RAG.</t>
   </si>
   <si>
-    <t>Authored Project Report Chapter 3: Data Ingestion Architecture, Multi-Format Parsing, and Chunking Algorithms.</t>
+    <t>Authored Project Report Chapter 3: Data Ingestion Architecture, Kaggle Dataset Extraction, and Chunking Algorithms.</t>
   </si>
   <si>
     <t>Authored Project Report Chapter 2: Literature Review, Theoretical Background on Vector Databases &amp; pgvector.</t>
@@ -1078,28 +1078,28 @@
     <t>Committed application screenshots and user guides to repository (3 commits).</t>
   </si>
   <si>
-    <t>Compiled all chapters into unified 65-page master Project Report document (3 commits).</t>
-  </si>
-  <si>
-    <t>Designed PPT Master Deck Slides 1-5 (Title, Problem Statement, Objectives, System Architecture, RAG Pipeline).</t>
-  </si>
-  <si>
-    <t>Designed PPT Slides 6-7 (Document Ingestion Engine, Recursive Chunking &amp; Apache Tika Pipeline).</t>
-  </si>
-  <si>
-    <t>Designed PPT Slides 8-9 (Neon Cloud Database, pgvector HNSW Indexing, Spring Security &amp; JWT).</t>
-  </si>
-  <si>
-    <t>Designed PPT Slides 10-11 (React UI Design, Electron Desktop Integration &amp; Streaming User Experience).</t>
-  </si>
-  <si>
-    <t>Designed PPT Slides 12-15 (Testing, JMeter Benchmarks, RAG Triad Evaluation Metrics &amp; Future Roadmap).</t>
+    <t>Compiled all chapters into unified master Project Report document (3 commits).</t>
+  </si>
+  <si>
+    <t>Designed PPT Master Deck Slides 1-3 (Title, Problem Statement, System Architecture, RAG Pipeline).</t>
+  </si>
+  <si>
+    <t>Designed PPT Slide 4 (Document Ingestion Engine, Recursive Chunking &amp; Apache Tika Pipeline).</t>
+  </si>
+  <si>
+    <t>Designed PPT Slide 5 (Neon Cloud Database, pgvector HNSW Indexing, Spring Security &amp; JWT).</t>
+  </si>
+  <si>
+    <t>Designed PPT Slide 6 (React UI Design, Electron Desktop Integration &amp; Streaming User Experience).</t>
+  </si>
+  <si>
+    <t>Designed PPT Slides 7-10 (Testing, JMeter Benchmarks, RAG Triad Evaluation Metrics &amp; Future Roadmap).</t>
   </si>
   <si>
     <t>Drafted 10-minute Demo Video script outlining speaking parts and feature demos for all 5 members.</t>
   </si>
   <si>
-    <t>Recorded screen capture segment demonstrating multi-format document upload and real-time chunking.</t>
+    <t>Recorded screen capture segment demonstrating multi-format document upload from Kaggle and real-time chunking.</t>
   </si>
   <si>
     <t>Recorded screen capture segment showing live Neon PostgreSQL console, pgvector queries, and JWT auth flow.</t>
@@ -1141,7 +1141,7 @@
     <t>Participated in mock viva; explained JMeter stress test graphs and error rates.</t>
   </si>
   <si>
-    <t>Presented PPT slides 1-5 to mentor Er. Ram Babu Buri during Saturday review.</t>
+    <t>Presented PPT deck to mentor Er. Ram Babu Buri during Saturday review.</t>
   </si>
   <si>
     <t>Reviewed ingestion demo clip and slides with mentor during Saturday review.</t>
@@ -1180,7 +1180,7 @@
     <t>Verified Neon PostgreSQL database production schema, connection quotas, and automated cloud backups.</t>
   </si>
   <si>
-    <t>Built Electron Windows installer (DocuQuery-AI-Setup-1.0.0.exe) using electron-builder.</t>
+    <t>Built Electron Windows installer using electron-builder.</t>
   </si>
   <si>
     <t>Conducted final regression testing on release v1.0.0 installer and backend JAR.</t>
@@ -1369,16 +1369,16 @@
     <t>2026-07-06 to 2026-07-11</t>
   </si>
   <si>
-    <t>https://github.com/aryankumarsingh/docuquery-rag/tree/main</t>
-  </si>
-  <si>
-    <t>Formed a 5-member team, finalized mentor Er. Ram Babu Buri. Defined problem statement: 'DocuQuery AI - Enterprise RAG Web &amp; Desktop System using Java Spring Boot, Neon PostgreSQL (pgvector), React/TS and Electron'. Divided into 5 distinct architectural modules. Prepared project abstract and registration.</t>
-  </si>
-  <si>
-    <t>Deciding between local Ollama embeddings vs cloud vector models and choosing between Swing vs Electron for modern desktop UI. Decided to adopt Spring Boot backend with hybrid React+Electron client.</t>
-  </si>
-  <si>
-    <t>Prepare Software Requirements Specification (SRS) in IEEE format and identify functional requirements for all 5 modules.</t>
+    <t>https://github.com/shauryadixit/docuquery-rag/tree/main</t>
+  </si>
+  <si>
+    <t>Formed 5-member team with guide Er. Ram Babu Buri. Finalized topic: 'DocuQuery AI: Enterprise RAG using Spring Boot, Neon pgvector, Electron, and Kaggle Research Corpus'. Partitioned into 5 distinct modules. Prepared project abstract.</t>
+  </si>
+  <si>
+    <t>Evaluating Kaggle multi-domain research paper dataset vs arXiv corpus for token size and formatting compatibility.</t>
+  </si>
+  <si>
+    <t>Formulate IEEE 830 Software Requirements Specification (SRS) for all 5 modules.</t>
   </si>
   <si>
     <t>Week 2</t>
@@ -1387,13 +1387,13 @@
     <t>2026-07-13 to 2026-07-18</t>
   </si>
   <si>
-    <t>Drafted and compiled complete Software Requirements Specification (SRS) following IEEE 830 standards. Specified functional requirements (FR1-FR15), non-functional requirements (performance, scalability, security, pgvector indexing), hardware/software requirements, and role-based permissions.</t>
-  </si>
-  <si>
-    <t>Defining latency constraints for LLM streaming responses over desktop Electron IPC while maintaining pgvector cosine similarity lookup under 150ms.</t>
-  </si>
-  <si>
-    <t>Design UML diagrams (Use Case, Class, Sequence, Component) reflecting system architecture and entity relationships.</t>
+    <t>Compiled complete IEEE 830 SRS document. Defined functional requirements FR1-FR15 (Kaggle dataset upload, chunking, pgvector search, JWT, SSE streaming) and non-functional requirements (latency, security, memory).</t>
+  </si>
+  <si>
+    <t>Defining latency constraints for 1536-dim vector searches over cloud Neon DB under 100ms.</t>
+  </si>
+  <si>
+    <t>Design UML diagrams (Use Case, Class, Sequence, Component, ER) for all modules.</t>
   </si>
   <si>
     <t>Week 3</t>
@@ -1402,13 +1402,13 @@
     <t>2026-07-20 to 2026-07-25</t>
   </si>
   <si>
-    <t>Constructed comprehensive UML models including System Use Case Diagram, Class Diagrams for Spring Boot domain and service layers, Sequence Diagrams for RAG Query and Document Ingestion pipelines, and Component/Deployment diagrams for Desktop-Cloud architecture.</t>
-  </si>
-  <si>
-    <t>Modeling the asynchronous streaming response between Spring Boot WebFlux/SSE and Electron IPC renderer without blocking the main event loop.</t>
-  </si>
-  <si>
-    <t>Design relational and vector database schemas in Neon PostgreSQL, construct UI interactive mockups in Figma/React.</t>
+    <t>Designed complete UML models: System Use Case Diagram, Class Diagram for Spring Boot entities and services, Sequence Diagrams for RAG Query and Kaggle Ingestion, Activity Diagram for chunking, and Component/ER models.</t>
+  </si>
+  <si>
+    <t>Modeling asynchronous streaming response between Spring Boot WebFlux and Electron IPC renderer.</t>
+  </si>
+  <si>
+    <t>Execute database DDL migrations on Neon PostgreSQL, setup HNSW index, initialize React+Vite project.</t>
   </si>
   <si>
     <t>Week 4</t>
@@ -1417,13 +1417,13 @@
     <t>2026-07-27 to 2026-08-01</t>
   </si>
   <si>
-    <t>Provisioned Neon PostgreSQL cloud instance, enabled pgvector extension, executed DDL scripts with HNSW index configuration. Built high-fidelity UI prototypes and initialized React 18 + TypeScript + Vite frontend project structure with Electron main/preload skeleton.</t>
-  </si>
-  <si>
-    <t>Tuning HNSW vector index parameters (m=16, ef_construction=64) on Neon PostgreSQL for optimal cosine distance search speed versus memory footprint.</t>
-  </si>
-  <si>
-    <t>Begin Module Coding Phase 1: Initialize Spring Boot project, configure build dependencies (Maven/Gradle), setup Git branches for all 5 members.</t>
+    <t>Configured Neon PostgreSQL cloud database, executed DDL migration scripts with HNSW index. Initialized React 18 + TypeScript + Vite frontend with Electron desktop shell. Downloaded Kaggle academic test corpus.</t>
+  </si>
+  <si>
+    <t>Tuning HNSW vector index parameters (m=16, ef_construction=64) on Neon for optimal lookup speed.</t>
+  </si>
+  <si>
+    <t>Begin Module Coding Phase 1: Initialize Spring Boot project, configure build dependencies, push initial commits.</t>
   </si>
   <si>
     <t>Week 5</t>
@@ -1435,10 +1435,10 @@
     <t>Implemented core RAG prompt formatting and query processing pipeline. Completed document parsing and recursive sliding-window chunking in Java. Implemented Spring Security JWT authentication and role-based filters. Built React chat message component.</t>
   </si>
   <si>
-    <t>Handling UTF-8 character encoding and ligatures in scanned PDF documents during Apache Tika extraction.</t>
-  </si>
-  <si>
-    <t>Implement vector embedding generation, store chunks in Neon pgvector, connect Electron frontend to Spring Boot REST endpoints.</t>
+    <t>Handling UTF-8 character encoding and ligatures in scanned PDF documents from Kaggle.</t>
+  </si>
+  <si>
+    <t>Implement vector embedding generation, store chunks in Neon pgvector, connect Electron frontend to Spring Boot.</t>
   </si>
   <si>
     <t>Week 6</t>
@@ -1447,10 +1447,10 @@
     <t>2026-08-10 to 2026-08-15</t>
   </si>
   <si>
-    <t>Connected document chunking pipeline to embedding generation service. Implemented batch insertion into Neon PostgreSQL using pgvector JDBC prepared statements. Built multipart file upload controller in Spring Boot and drag-and-drop file uploader in React.</t>
-  </si>
-  <si>
-    <t>Batch inserting large vectors (1536 float dimensions) caused memory spikes; resolved by implementing batched paging of 50 chunks per transaction.</t>
+    <t>Connected Kaggle document chunking pipeline to embedding generation service. Implemented batch insertion into Neon PostgreSQL using pgvector JDBC prepared statements. Built multipart file upload controller in Spring Boot and drag-and-drop file uploader in React.</t>
+  </si>
+  <si>
+    <t>Batch inserting large vectors caused memory spikes; resolved by implementing batched paging of 50 chunks.</t>
   </si>
   <si>
     <t>Implement Server-Sent Events (SSE) streaming chat API and connect Electron frontend to streaming endpoint.</t>
@@ -1462,7 +1462,7 @@
     <t>2026-08-17 to 2026-08-22</t>
   </si>
   <si>
-    <t>Implemented Server-Sent Events (SSE) streaming API (/api/rag/chat/stream) delivering token-by-token LLM responses. Implemented dynamic source citation referencing linking generated statements to exact document chunks and page numbers. Integrated desktop native notifications in Electron.</t>
+    <t>Implemented Server-Sent Events (SSE) streaming API (/api/rag/chat/stream) delivering token-by-token LLM responses. Implemented dynamic source citation referencing linking generated statements to exact Kaggle paper excerpts. Integrated desktop native notifications in Electron.</t>
   </si>
   <si>
     <t>Handling client disconnection mid-stream and ensuring LLM stream cancels promptly to conserve compute tokens.</t>
@@ -1477,7 +1477,7 @@
     <t>2026-08-24 to 2026-08-29</t>
   </si>
   <si>
-    <t>Built automated RAG Triad evaluation service measuring Context Relevance, Faithfulness, and Answer Relevance. Created Admin Analytics Dashboard in React displaying real-time query latency, token usage graphs, index size, and user activity metrics.</t>
+    <t>Built automated RAG Triad evaluation service measuring Context Relevance, Faithfulness, and Answer Relevance against Kaggle ground-truth questions. Created Admin Analytics Dashboard in React displaying real-time query latency and token usage graphs.</t>
   </si>
   <si>
     <t>Formulating a cost-effective evaluation metric that calculates faithfulness without incurring high extra LLM API latency.</t>
@@ -1537,7 +1537,7 @@
     <t>2026-09-21 to 2026-09-26</t>
   </si>
   <si>
-    <t>Created 15-slide PowerPoint (PPT) presentation deck. Recorded 10-minute HD demo video showcasing live system architecture, document upload, pgvector similarity search, token-by-token streaming, source citations, and admin analytics. Conducted mock viva voce sessions.</t>
+    <t>Created 10-slide PowerPoint (PPT) presentation deck. Recorded 10-minute HD demo video showcasing live system architecture, Kaggle document upload, pgvector similarity search, token-by-token streaming, source citations, and admin analytics. Conducted mock viva voce sessions.</t>
   </si>
   <si>
     <t>Recording demo video with clean audio and demonstrating both local Electron desktop window and Neon cloud database queries simultaneously.</t>
@@ -1603,7 +1603,7 @@
     <t>RAG retrieval controller, prompt engineering, token streaming SSE, hallucination guardrails</t>
   </si>
   <si>
-    <t>Data Engineer &amp; Document Processing Lead</t>
+    <t>Data Engineer &amp; Kaggle Ingestion Lead</t>
   </si>
   <si>
     <t>feature/member2-doc-ingestion</t>
@@ -1612,7 +1612,7 @@
     <t>Apache Tika, Apache PDFBox 3, JTokkit, Spring Async</t>
   </si>
   <si>
-    <t>Multi-format parser (PDF, DOCX, TXT), recursive sliding-window chunker, multipart upload worker</t>
+    <t>Kaggle research paper parser (PDF, DOCX, TXT), recursive sliding chunker, multipart upload worker</t>
   </si>
   <si>
     <t>Database Architect &amp; Security Engineer</t>
@@ -1642,16 +1642,13 @@
     <t>QA, RAG Evaluation &amp; Analytics Lead</t>
   </si>
   <si>
-    <t>Module 5: RAG Triad Evaluation, Performance Analytics &amp; Admin Dashboard</t>
-  </si>
-  <si>
     <t>feature/member5-analytics-evaluation</t>
   </si>
   <si>
     <t>JUnit 5, Mockito, Apache JMeter, Recharts, JaCoCo</t>
   </si>
   <si>
-    <t>RAG Triad evaluation metrics (Faithfulness/Relevance), JMeter load tests, Admin telemetry dashboard</t>
+    <t>RAG Triad evaluation metrics (Faithfulness/Relevance on Kaggle dataset), JMeter load tests, Admin telemetry dashboard</t>
   </si>
 </sst>
 </file>
@@ -2052,13 +2049,13 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E24F4C25-DA04-4DEE-8A03-D6A85126C579}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE925B36-C6F8-42C4-930F-B290A1EDACF1}">
   <dimension ref="A1:F421"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="49.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="55.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.77734375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="128" bestFit="1" customWidth="1"/>
@@ -10486,22 +10483,21 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF81E045-B2AF-41FE-8CA3-B082846BA341}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74B480B7-82AF-41CF-B733-030712923DBC}">
   <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="52.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="48" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="253.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="165.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="117.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="144.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="104.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -10855,16 +10851,16 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F53B4BED-0C21-4C45-BD2B-BC2574145127}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFF34ECF-B905-4C6D-B059-0981AB69652D}">
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="36.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="62" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="55.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="32.44140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="56.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="83.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="97.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
@@ -10975,16 +10971,16 @@
         <v>533</v>
       </c>
       <c r="C6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" t="s">
         <v>534</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>535</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>536</v>
-      </c>
-      <c r="F6" t="s">
-        <v>537</v>
       </c>
     </row>
   </sheetData>

</xml_diff>